<commit_message>
verify CLS batch 1: 7 ImageNet-1K Top-1 fills from MambaVision Table 1
Filled from MambaVision (arXiv 2407.08083) Table 1 comprehensive comparison:
- MambaVision-S: 83.3   - MambaVision-T: 82.3
- VMamba-S:      83.6   - VMamba-T:      82.6
- Vim-T:         76.1   - Vim-S:         80.5
- EfficientNetV2-S: 83.9

CLS verified: 0 → 7; unverified: 221 → 214.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Image_Classification_Papers_Ranking_2021_2026.xlsx
+++ b/Image_Classification_Papers_Ranking_2021_2026.xlsx
@@ -583,7 +583,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O114"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -9247,7 +9247,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -10307,7 +10307,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -11208,7 +11208,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -12692,7 +12692,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -14385,7 +14385,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -16186,7 +16186,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -18093,7 +18093,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -18992,7 +18992,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -19893,7 +19893,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -20794,7 +20794,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -21695,7 +21695,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O103"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -24262,15 +24262,23 @@
           <t>預印本</t>
         </is>
       </c>
-      <c r="G34" s="3" t="n"/>
+      <c r="G34" s="3" t="n">
+        <v>83.3</v>
+      </c>
       <c r="H34" s="3" t="n"/>
-      <c r="I34" s="3" t="n"/>
+      <c r="I34" s="3" t="n">
+        <v>83.3</v>
+      </c>
       <c r="J34" s="3" t="n"/>
-      <c r="K34" s="3" t="n"/>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>50.1M</t>
+        </is>
+      </c>
       <c r="L34" s="3" t="n"/>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>⚠️ 自動抽取・指標待驗證 (已偵測使用此資料集)：Hybrid Mamba+Transformer; small variant</t>
+          <t>✅ 已驗證 (MambaVision Table 1, ImageNet-1K)：MambaVision-S Top-1 83.3% [Mamba-based]</t>
         </is>
       </c>
       <c r="N34" s="4" t="inlineStr">
@@ -24315,15 +24323,23 @@
           <t>預印本</t>
         </is>
       </c>
-      <c r="G35" s="3" t="n"/>
+      <c r="G35" s="3" t="n">
+        <v>82.3</v>
+      </c>
       <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n"/>
+      <c r="I35" s="3" t="n">
+        <v>82.3</v>
+      </c>
       <c r="J35" s="3" t="n"/>
-      <c r="K35" s="3" t="n"/>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>31.8M</t>
+        </is>
+      </c>
       <c r="L35" s="3" t="n"/>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>⚠️ 自動抽取・指標待驗證 (已偵測使用此資料集)：Hybrid Mamba+Transformer; tiny variant</t>
+          <t>✅ 已驗證 (MambaVision Table 1, ImageNet-1K)：MambaVision-T Top-1 82.3% [Mamba-based]</t>
         </is>
       </c>
       <c r="N35" s="4" t="inlineStr">
@@ -24368,15 +24384,23 @@
           <t>預印本</t>
         </is>
       </c>
-      <c r="G36" s="3" t="n"/>
+      <c r="G36" s="3" t="n">
+        <v>83.59999999999999</v>
+      </c>
       <c r="H36" s="3" t="n"/>
-      <c r="I36" s="3" t="n"/>
+      <c r="I36" s="3" t="n">
+        <v>83.59999999999999</v>
+      </c>
       <c r="J36" s="3" t="n"/>
-      <c r="K36" s="3" t="n"/>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>50.0M</t>
+        </is>
+      </c>
       <c r="L36" s="3" t="n"/>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>⚠️ 自動抽取・指標待驗證 (已偵測使用此資料集)：VMamba small</t>
+          <t>✅ 已驗證 (MambaVision Table 1, ImageNet-1K)：VMamba-S Top-1 83.6% [Mamba-based]</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
@@ -24421,15 +24445,23 @@
           <t>預印本</t>
         </is>
       </c>
-      <c r="G37" s="3" t="n"/>
+      <c r="G37" s="3" t="n">
+        <v>82.59999999999999</v>
+      </c>
       <c r="H37" s="3" t="n"/>
-      <c r="I37" s="3" t="n"/>
+      <c r="I37" s="3" t="n">
+        <v>82.59999999999999</v>
+      </c>
       <c r="J37" s="3" t="n"/>
-      <c r="K37" s="3" t="n"/>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>30.0M</t>
+        </is>
+      </c>
       <c r="L37" s="3" t="n"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>⚠️ 自動抽取・指標待驗證 (已偵測使用此資料集)：VMamba tiny</t>
+          <t>✅ 已驗證 (MambaVision Table 1, ImageNet-1K)：VMamba-T Top-1 82.6% [Mamba-based]</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -24580,15 +24612,23 @@
           <t>預印本</t>
         </is>
       </c>
-      <c r="G40" s="3" t="n"/>
+      <c r="G40" s="3" t="n">
+        <v>76.09999999999999</v>
+      </c>
       <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="n"/>
+      <c r="I40" s="3" t="n">
+        <v>76.09999999999999</v>
+      </c>
       <c r="J40" s="3" t="n"/>
-      <c r="K40" s="3" t="n"/>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>7.0M</t>
+        </is>
+      </c>
       <c r="L40" s="3" t="n"/>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>⚠️ 自動抽取・指標待驗證 (已偵測使用此資料集)：Vision Mamba bidirectional SSM tiny</t>
+          <t>✅ 已驗證 (MambaVision Table 1, ImageNet-1K)：Vim-T Top-1 76.1% [Mamba-based]</t>
         </is>
       </c>
       <c r="N40" s="4" t="inlineStr">
@@ -24633,15 +24673,23 @@
           <t>預印本</t>
         </is>
       </c>
-      <c r="G41" s="3" t="n"/>
+      <c r="G41" s="3" t="n">
+        <v>80.5</v>
+      </c>
       <c r="H41" s="3" t="n"/>
-      <c r="I41" s="3" t="n"/>
+      <c r="I41" s="3" t="n">
+        <v>80.5</v>
+      </c>
       <c r="J41" s="3" t="n"/>
-      <c r="K41" s="3" t="n"/>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>26.0M</t>
+        </is>
+      </c>
       <c r="L41" s="3" t="n"/>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>⚠️ 自動抽取・指標待驗證 (已偵測使用此資料集)：Vision Mamba small</t>
+          <t>✅ 已驗證 (MambaVision Table 1, ImageNet-1K)：Vim-S Top-1 80.5% [Mamba-based]</t>
         </is>
       </c>
       <c r="N41" s="4" t="inlineStr">
@@ -26382,15 +26430,23 @@
           <t>預印本</t>
         </is>
       </c>
-      <c r="G74" s="3" t="n"/>
+      <c r="G74" s="3" t="n">
+        <v>83.90000000000001</v>
+      </c>
       <c r="H74" s="3" t="n"/>
-      <c r="I74" s="3" t="n"/>
+      <c r="I74" s="3" t="n">
+        <v>83.90000000000001</v>
+      </c>
       <c r="J74" s="3" t="n"/>
-      <c r="K74" s="3" t="n"/>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>21.5M</t>
+        </is>
+      </c>
       <c r="L74" s="3" t="n"/>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>⚠️ 自動抽取・指標待驗證 (已偵測使用此資料集)：EfficientNetV2-S</t>
+          <t>✅ 已驗證 (MambaVision Table 1, ImageNet-1K)：EfficientNetV2-S Top-1 83.9% [Conv-based]</t>
         </is>
       </c>
       <c r="N74" s="4" t="inlineStr">
@@ -28018,7 +28074,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -28919,7 +28975,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -29978,7 +30034,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -30879,7 +30935,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -31780,7 +31836,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -32680,7 +32736,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -33580,7 +33636,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -35010,7 +35066,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -36069,7 +36125,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -36970,7 +37026,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -37871,7 +37927,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -39567,7 +39623,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -40468,7 +40524,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -41369,7 +41425,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -42270,7 +42326,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -43171,7 +43227,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -44072,7 +44128,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -44973,7 +45029,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -45874,7 +45930,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -46775,7 +46831,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -47676,7 +47732,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -48577,7 +48633,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -50856,7 +50912,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O48"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>

</xml_diff>